<commit_message>
docs: update release evidence candidate
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="407">
   <si>
     <t xml:space="preserve">Codomyrmex Review Action Register</t>
   </si>
   <si>
-    <t xml:space="preserve">Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Candidate evidence 14 July 2026</t>
+    <t xml:space="preserve">Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Implementation candidate 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025 | Evidence 14 July 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Open blockers</t>
@@ -701,7 +701,7 @@
     <t xml:space="preserve">Evidence summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Current revision evidence (4bd6c1804f2c)</t>
+    <t xml:space="preserve">Current candidate evidence (1db2b7a326b4)</t>
   </si>
   <si>
     <t xml:space="preserve">Attached PDF: 50 pages, SHA-256 c1432347b75c34258fb53d29b4d747684fbc06655126fd5af37182b0928a4270. Public main at e85aee6758726ca1fbba202d0ef1a09d524029e3 contains a 77-page output/paper.pdf, SHA-256 6333fde6bd65aa25406ce5491424010ec5b15f932093e3ea64954d91f0a7723d. Public 02_methodology.md says FAILURE does not directly reduce risk_ok, while the attachment says max(RISK, FAILURE); the public abstract also retains stronger persistence/control claims.</t>
@@ -710,33 +710,57 @@
     <t xml:space="preserve">The attachment states effective hazard = max(RISK, FAILURE) and reports 0.875/EXECUTE -&gt; 0.725/HOLD after a same-target FAILURE. Public actuation_gate.py reads witness state but assigns risk_pressure = pheromone_readings['risk']; direct replay produced 0.875/EXECUTE before, FAILURE pressure 3.0, 0.875/EXECUTE afterward, and 0.875/EXECUTE at an unrelated target.</t>
   </si>
   <si>
+    <t xml:space="preserve">Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Attachment reports 773 passing tests and 78.7% branch coverage. Public main produced 764 collected, 763 passed, 1 skipped, and 475/606 branches covered = 78.382838...%, reported as 78.4%. Ruff and ty both reproduced at zero.</t>
   </si>
   <si>
+    <t xml:space="preserve">Fresh candidate run: 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; branch 74.10714285714286% (581/784); line 82.44274809160305% (2,227/2,622); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">The attachment instructs ./run.sh --pipeline --project ongoing/codomyrmex --core-only and then cd projects/ongoing/codomyrmex. Public main contains neither run.sh nor projects/ongoing/codomyrmex.</t>
   </si>
   <si>
     <t xml:space="preserve">ActuationGate applies the &gt;=3-failure penalty only when self._memory is non-null. ColonyKernel constructs ActuationGate(pheromone_store=...) and constructs ConsequenceMemory separately, never passing consequence_memory_ref.</t>
   </si>
   <si>
+    <t xml:space="preserve">ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ActuationGate evaluates bool(self._ledger.can_afford(...)); ResourceLedger.can_afford returns a tuple. bool((False, reason)) is True. With max_llm_calls=0 and an estimate of 1, the ledger returned (False, reason) but the standalone gate returned 0.875/EXECUTE and budget_approved=True.</t>
   </si>
   <si>
+    <t xml:space="preserve">Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">FalsificationWorker.analyze maps target, rationale, rollback_plan, evidence, action_type and budget_estimate, but omits expected_outcome and other plan semantics used by checks. A complete ActionProposal can therefore acquire findings unrelated to its actual completeness. In the canonical path, four adapter-driven findings deposited RISK 3.0 and produced 0.725/HOLD at both the target and an otherwise clear unrelated target; HIGH/CRITICAL findings can also deposit pre-execution FAILURE.</t>
   </si>
   <si>
+    <t xml:space="preserve">ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ColonyKernel.propose_action deposits FAILURE for every REFUSE, and FalsificationWorker deposits FAILURE for HIGH/CRITICAL prospective findings before a gate decision or execution. Under max(RISK, FAILURE), either path can manufacture the pressure that drives subsequent refusal.</t>
   </si>
   <si>
     <t xml:space="preserve">colony_record_outcome accepts agent_id/action_type/target/text/tests_passed, synthesizes a new ActionProposal, and explicitly does not require the original proposal_id. No EXECUTE verdict, caller identity, authorization, test attestation, deduplication or target binding is verified.</t>
   </si>
   <si>
+    <t xml:space="preserve">Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">The proposal MCP tool returns a serialized GateResult but issues no authorization token and has no downstream action executor or consumed capability. Callers can ignore the result.</t>
   </si>
   <si>
+    <t xml:space="preserve">Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">At the pinned revision, only src/codomyrmex/cli/doctor.py instantiates ColonyKernel outside its own package. A tracked-source scan found 630 actual @mcp_tool decorator definitions (653 textual occurrences) repo-wide and 8 in colony_kernel; the other tool paths are not routed through the gate. Colony AGENTS.md says it 'gates every agent action.'</t>
   </si>
   <si>
+    <t xml:space="preserve">Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+  </si>
+  <si>
     <t xml:space="preserve">New agents start at trust 0.10/SANDBOX and cannot pass write-path gating. Tests promote agents by directly calling record_outcome with constructed successful proposals, bypassing the gate and any attestation. Three such reports reach trust 0.22 and REPAIR_ANT, still below the 0.30 gate floor.</t>
   </si>
   <si>
@@ -821,7 +845,7 @@
     <t xml:space="preserve">Full Git SHA, clean status, dependency lock hash, config digest and source archive are recorded.</t>
   </si>
   <si>
-    <t xml:space="preserve">Manifest records HEAD 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837, dirty state, lock/config/source hashes, tools, and artifact hashes; clean immutable tag pending.</t>
+    <t xml:space="preserve">Manifest candidate records implementation revision 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025, lock/config/source hashes, tools, status, and artifact hashes; local unrelated changes remain outside the candidate; immutable tag pending.</t>
   </si>
   <si>
     <t xml:space="preserve">R-02</t>
@@ -836,7 +860,7 @@
     <t xml:space="preserve">Manuscript/release</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidate PDF rendered with 0.20-inch side margins; SHA-256 2f6f10e2cac4ac357003cc278a86242806a660e6167dcb95da71983b2993c6e8. Clean-clone byte/hash replay remains pending.</t>
+    <t xml:space="preserve">Canonical PDF SHA-256 36ebc8982f92d5bd007b92f9415d029dfc26ee4c5aa185c0345fc8b48b1f0f76; clean clone at 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025 regenerated the exact PDF, HTML, and figure hashes with SOURCE_DATE_EPOCH pinning; immutable tag pending.</t>
   </si>
   <si>
     <t xml:space="preserve">R-03</t>
@@ -848,7 +872,7 @@
     <t xml:space="preserve">The manuscript, source, tests, generated variables and rendered artifacts all come from the same tagged revision.</t>
   </si>
   <si>
-    <t xml:space="preserve">Source, generated variables, coverage, JUnit, HTML, PDF, and release manifest were regenerated from one candidate worktree; immutable tag pending.</t>
+    <t xml:space="preserve">Candidate source, variables, coverage, JUnit, HTML, PDF, and figures were regenerated at 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025; clean-clone hashes match; immutable tag pending.</t>
   </si>
   <si>
     <t xml:space="preserve">R-04</t>
@@ -1019,7 +1043,7 @@
     <t xml:space="preserve">Independent reviewer</t>
   </si>
   <si>
-    <t xml:space="preserve">Independent clean-checkout replay and immutable release/tag are the remaining publication blocker.</t>
+    <t xml:space="preserve">Clean-clone replay at 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025 passed with exact PDF/HTML/figure hashes; independent reviewer confirmation and immutable tag remain.</t>
   </si>
   <si>
     <t xml:space="preserve">R-16</t>
@@ -1079,7 +1103,7 @@
     <t xml:space="preserve">Colony Kernel/security</t>
   </si>
   <si>
-    <t xml:space="preserve">Real-component lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, and quarantine contracts pass; clean-clone verification pending.</t>
+    <t xml:space="preserve">Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay also passes.</t>
   </si>
   <si>
     <t xml:space="preserve">R-20</t>
@@ -1109,19 +1133,19 @@
     <t xml:space="preserve">Current evaluated revision</t>
   </si>
   <si>
-    <t xml:space="preserve">4bd6c1804f2caa905d36bcb39d67bdf8c1d86837</t>
+    <t xml:space="preserve">1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025</t>
   </si>
   <si>
     <t xml:space="preserve">Release tag</t>
   </si>
   <si>
-    <t xml:space="preserve">Pending clean immutable release</t>
+    <t xml:space="preserve">Pending immutable v1.4.0-rc1 tag; clean-clone replay verified at implementation candidate</t>
   </si>
   <si>
     <t xml:space="preserve">Publication manifest</t>
   </si>
   <si>
-    <t xml:space="preserve">publication_ready=false; dirty worktree; required test/artifact gates fresh; provider benchmark missing</t>
+    <t xml:space="preserve">publication_ready=false; local unrelated worktree changes; required test/artifact gates fresh; provider benchmark missing</t>
   </si>
   <si>
     <t xml:space="preserve">Required tests</t>
@@ -1133,7 +1157,7 @@
     <t xml:space="preserve">Coverage</t>
   </si>
   <si>
-    <t xml:space="preserve">74.10714285714286% (581/784) branch; 82.44274809160305% (2,227/2,622) line; floor 60.0%</t>
+    <t xml:space="preserve">74.29667519181585% (581/782) branch; 82.57419923596827% (2,229/2,621) line; floor 60.0%</t>
   </si>
   <si>
     <t xml:space="preserve">Locality</t>
@@ -1151,13 +1175,13 @@
     <t xml:space="preserve">Canonical PDF SHA-256</t>
   </si>
   <si>
-    <t xml:space="preserve">2f6f10e2cac4ac357003cc278a86242806a660e6167dcb95da71983b2993c6e8</t>
+    <t xml:space="preserve">36ebc8982f92d5bd007b92f9415d029dfc26ee4c5aa185c0345fc8b48b1f0f76</t>
   </si>
   <si>
     <t xml:space="preserve">Manifest SHA-256</t>
   </si>
   <si>
-    <t xml:space="preserve">aa336607eb304523b279a367eedf671218fe15fe017a444ca27e6357ff50b7e2</t>
+    <t xml:space="preserve">Pending final manifest regeneration after immutable tag</t>
   </si>
   <si>
     <t xml:space="preserve">Artifact</t>
@@ -1169,37 +1193,34 @@
     <t xml:space="preserve">output/paper.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">5aa7baf44254249f3ee7fe6130147ea6754d8f38089cc5f8aaf390e1e5660ff7</t>
-  </si>
-  <si>
     <t xml:space="preserve">output/paper.html</t>
   </si>
   <si>
-    <t xml:space="preserve">364245b2662000d8b1a4c11fdffaf2c9006e15ef9c0df57591e6d01fe653baae</t>
+    <t xml:space="preserve">6d999977449e85e979992f07c16472bdea07e5ab8e8018ce34a421e0938120df</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/manuscript_variables.json</t>
   </si>
   <si>
-    <t xml:space="preserve">935cdf16bbb05257a0efd4c778d9c25a4b6d724c8f6ede570f63bca36a4049e5</t>
+    <t xml:space="preserve">6b424188e10d340dce60cb520809ab30ab3014fb9681b7935befa63271b86c98</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_coverage.json</t>
   </si>
   <si>
-    <t xml:space="preserve">ea8436096c3fd8da6e88e1ea055f262a03ee052e54ad4cd201017b2120f6461b</t>
+    <t xml:space="preserve">117dcb7145d1455a2f0125e954c92ff016012622e7e1f6a951b26996541cceb2</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_test_report.xml</t>
   </si>
   <si>
-    <t xml:space="preserve">d20f76c362548c392eba1a3995634611d5bae14770e7ce0f386ec3bed5ea4a74</t>
+    <t xml:space="preserve">0dad5f0f470c4bf770bf7bb3f15169099113e4e28a8f6af203caf232c7102355</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_test_status.json</t>
   </si>
   <si>
-    <t xml:space="preserve">0b1067d4ba8fa86aa895eaeaad1a01fd24d254a00897eae11980a062fd3a2ea0</t>
+    <t xml:space="preserve">abe20b74d40742d444770bc68e96979f916c8766971eaca62759d01ee12657af</t>
   </si>
   <si>
     <t xml:space="preserve">output/release_manifest.json</t>
@@ -1211,7 +1232,7 @@
     <t xml:space="preserve">Enforcement profile</t>
   </si>
   <si>
-    <t xml:space="preserve">Strict declared-scope capabilities and receipts implemented; advisory compatibility retained</t>
+    <t xml:space="preserve">Strict declared-scope Ed25519 capabilities and receipts implemented; advisory compatibility retained</t>
   </si>
   <si>
     <t xml:space="preserve">SWE-bench Lite pin</t>
@@ -2423,11 +2444,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="6495430"/>
-        <c:axId val="60677435"/>
+        <c:axId val="75438293"/>
+        <c:axId val="54312665"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="6495430"/>
+        <c:axId val="75438293"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2472,7 +2493,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60677435"/>
+        <c:crossAx val="54312665"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2480,7 +2501,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60677435"/>
+        <c:axId val="54312665"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2525,7 +2546,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6495430"/>
+        <c:crossAx val="75438293"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2781,9 +2802,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>983520</xdr:colOff>
+      <xdr:colOff>983160</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>187200</xdr:rowOff>
+      <xdr:rowOff>186840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2792,7 +2813,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4299480" y="1609560"/>
-        <a:ext cx="4930920" cy="3425760"/>
+        <a:ext cx="4930560" cy="3425400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4501,7 +4522,7 @@
         <v>227</v>
       </c>
       <c r="D6" s="41" t="s">
-        <v>52</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4512,10 +4533,10 @@
         <v>54</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>58</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4526,7 +4547,7 @@
         <v>60</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D8" s="41" t="s">
         <v>63</v>
@@ -4540,10 +4561,10 @@
         <v>65</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D9" s="41" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4554,10 +4575,10 @@
         <v>70</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D10" s="41" t="s">
-        <v>73</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4568,10 +4589,10 @@
         <v>75</v>
       </c>
       <c r="C11" s="40" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D11" s="41" t="s">
-        <v>79</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4582,7 +4603,7 @@
         <v>82</v>
       </c>
       <c r="C12" s="40" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D12" s="41" t="s">
         <v>86</v>
@@ -4596,10 +4617,10 @@
         <v>88</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="D13" s="41" t="s">
-        <v>92</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4610,10 +4631,10 @@
         <v>95</v>
       </c>
       <c r="C14" s="40" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="D14" s="41" t="s">
-        <v>99</v>
+        <v>242</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4624,10 +4645,10 @@
         <v>101</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>105</v>
+        <v>244</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4638,7 +4659,7 @@
         <v>107</v>
       </c>
       <c r="C16" s="40" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D16" s="41" t="s">
         <v>111</v>
@@ -4652,7 +4673,7 @@
         <v>113</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="D17" s="41" t="s">
         <v>117</v>
@@ -4666,7 +4687,7 @@
         <v>119</v>
       </c>
       <c r="C18" s="40" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="D18" s="41" t="s">
         <v>123</v>
@@ -4680,7 +4701,7 @@
         <v>125</v>
       </c>
       <c r="C19" s="40" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D19" s="41" t="s">
         <v>129</v>
@@ -4694,7 +4715,7 @@
         <v>131</v>
       </c>
       <c r="C20" s="40" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D20" s="41" t="s">
         <v>135</v>
@@ -4708,7 +4729,7 @@
         <v>137</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="D21" s="41" t="s">
         <v>141</v>
@@ -4722,7 +4743,7 @@
         <v>143</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D22" s="41" t="s">
         <v>147</v>
@@ -4736,7 +4757,7 @@
         <v>149</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D23" s="41" t="s">
         <v>153</v>
@@ -4750,7 +4771,7 @@
         <v>155</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D24" s="41" t="s">
         <v>159</v>
@@ -4764,7 +4785,7 @@
         <v>161</v>
       </c>
       <c r="C25" s="40" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D25" s="41" t="s">
         <v>165</v>
@@ -4778,7 +4799,7 @@
         <v>167</v>
       </c>
       <c r="C26" s="40" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="D26" s="41" t="s">
         <v>171</v>
@@ -4792,7 +4813,7 @@
         <v>173</v>
       </c>
       <c r="C27" s="40" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="D27" s="41" t="s">
         <v>176</v>
@@ -4806,7 +4827,7 @@
         <v>178</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D28" s="41" t="s">
         <v>181</v>
@@ -4820,7 +4841,7 @@
         <v>183</v>
       </c>
       <c r="C29" s="40" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="D29" s="41" t="s">
         <v>187</v>
@@ -4834,7 +4855,7 @@
         <v>189</v>
       </c>
       <c r="C30" s="40" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="D30" s="41" t="s">
         <v>192</v>
@@ -4848,7 +4869,7 @@
         <v>194</v>
       </c>
       <c r="C31" s="40" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="D31" s="41" t="s">
         <v>198</v>
@@ -4862,7 +4883,7 @@
         <v>200</v>
       </c>
       <c r="C32" s="40" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="D32" s="41" t="s">
         <v>204</v>
@@ -4876,7 +4897,7 @@
         <v>206</v>
       </c>
       <c r="C33" s="40" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="D33" s="41" t="s">
         <v>209</v>
@@ -4890,7 +4911,7 @@
         <v>211</v>
       </c>
       <c r="C34" s="40" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="D34" s="41" t="s">
         <v>214</v>
@@ -4904,7 +4925,7 @@
         <v>216</v>
       </c>
       <c r="C35" s="40" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="D35" s="41" t="s">
         <v>220</v>
@@ -4946,7 +4967,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4956,7 +4977,7 @@
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4969,10 +4990,10 @@
         <v>33</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>38</v>
@@ -4981,18 +5002,18 @@
         <v>16</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="38" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="B5" s="40" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D5" s="40" t="s">
         <v>134</v>
@@ -5001,38 +5022,38 @@
         <v>22</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="38" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="D6" s="40" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="E6" s="39" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="38" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="D7" s="40" t="s">
         <v>134</v>
@@ -5041,347 +5062,347 @@
         <v>22</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="D8" s="40" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="E8" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="41" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="D9" s="40" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="E9" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="41" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="C10" s="40" t="s">
+        <v>294</v>
+      </c>
+      <c r="D10" s="40" t="s">
         <v>286</v>
-      </c>
-      <c r="D10" s="40" t="s">
-        <v>278</v>
       </c>
       <c r="E10" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="41" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="C11" s="40" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="E11" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F11" s="41" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C12" s="40" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="E12" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F12" s="41" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="38" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="B13" s="40" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="E13" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="38" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="B14" s="40" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="C14" s="40" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="E14" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F14" s="41" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="38" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="D15" s="40" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="E15" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="38" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="C16" s="40" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="D16" s="40" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="E16" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F16" s="41" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="38" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="D17" s="40" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="E17" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="41" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="38" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="C18" s="40" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="D18" s="40" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="E18" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F18" s="41" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="38" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="C19" s="40" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="D19" s="40" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="E19" s="39" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F19" s="41" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="38" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="C20" s="40" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="D20" s="40" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="38" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="D21" s="40" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="E21" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F21" s="41" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="38" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="B22" s="40" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="D22" s="40" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E22" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F22" s="41" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="38" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B23" s="40" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="D23" s="40" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="E23" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F23" s="41" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="38" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D24" s="40" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="E24" s="39" t="s">
         <v>18</v>
       </c>
       <c r="F24" s="41" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -5434,7 +5455,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="42" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -5442,172 +5463,172 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="43" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="43" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="43" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="45" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B15" s="45" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="45"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="B16" s="46" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="B17" s="46" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="B18" s="46" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B19" s="46" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="B20" s="46" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="B21" s="46" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="B22" s="46" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="B23" s="46" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="B24" s="46" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="B25" s="46" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: finalize rc1 provenance
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="408">
   <si>
     <t xml:space="preserve">Codomyrmex Review Action Register</t>
   </si>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Current recommendation</t>
   </si>
   <si>
-    <t xml:space="preserve">PUBLICATION HOLD. A-002/A-003/A-005/A-006 are fixed in the current revision pending clean-release verification; A-001 and A-016 remain release blockers until the exact PDF-producing source and evidence bundle are committed and tagged.</t>
+    <t xml:space="preserve">PUBLICATION HOLD. A-002/A-003/A-005/A-006 are verified in the v1.4.0-rc1 candidate; A-001 and A-016 remain open until the candidate evidence is externally published and the provider benchmark is complete.</t>
   </si>
   <si>
     <t xml:space="preserve">Source package: consolidated two-pass report and reproduction evidence. Public repository: https://github.com/docxology/codomyrmex/commit/e85aee6758726ca1fbba202d0ef1a09d524029e3</t>
@@ -164,7 +164,7 @@
     <t xml:space="preserve">Daniel + release maintainer</t>
   </si>
   <si>
-    <t xml:space="preserve">Still open: manifest publication_ready=false because the candidate worktree is dirty and untagged. Clean-clone replay and immutable release remain required.</t>
+    <t xml:space="preserve">Candidate is committed and tagged v1.4.0-rc1; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
   </si>
   <si>
     <t xml:space="preserve">A-002</t>
@@ -776,6 +776,9 @@
     <t xml:space="preserve">git ls-files output lists only output/paper.html and output/paper.pdf. Generated manuscript_variables.json, colony_kernel_coverage.json and expanded manuscript files are ignored. figure_registry.json and output/figures were absent in the audit checkout.</t>
   </si>
   <si>
+    <t xml:space="preserve">Candidate evidence and the clean-clone release package exist with PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
+  </si>
+  <si>
     <t xml:space="preserve">The critical/high FAILURE-pressure tests seed only three direct successes, yielding trust 0.22, which is below the separate 0.30 hard floor. REFUSE can therefore occur because of trust, and broad assertions such as HOLD-or-REFUSE do not prove the pressure mechanism.</t>
   </si>
   <si>
@@ -845,7 +848,7 @@
     <t xml:space="preserve">Full Git SHA, clean status, dependency lock hash, config digest and source archive are recorded.</t>
   </si>
   <si>
-    <t xml:space="preserve">Manifest candidate records implementation revision f22384acf925cebdd819915d17d530592d9ffba3, lock/config/source hashes, tools, status, and artifact hashes; local unrelated changes remain outside the candidate; immutable tag pending.</t>
+    <t xml:space="preserve">Manifest records the v1.4.0-rc1 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
   </si>
   <si>
     <t xml:space="preserve">R-02</t>
@@ -860,7 +863,7 @@
     <t xml:space="preserve">Manuscript/release</t>
   </si>
   <si>
-    <t xml:space="preserve">Canonical PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2; clean clone at f22384acf925cebdd819915d17d530592d9ffba3 regenerated the exact PDF, HTML, and figure hashes with SOURCE_DATE_EPOCH pinning; immutable tag pending.</t>
+    <t xml:space="preserve">Canonical PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2; clean clone at tagged v1.4.0-rc1 regenerated the exact PDF, HTML, evidence, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
   </si>
   <si>
     <t xml:space="preserve">R-03</t>
@@ -872,7 +875,7 @@
     <t xml:space="preserve">The manuscript, source, tests, generated variables and rendered artifacts all come from the same tagged revision.</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidate source, variables, coverage, JUnit, HTML, PDF, and figures were regenerated at f22384acf925cebdd819915d17d530592d9ffba3; clean-clone hashes match; immutable tag pending.</t>
+    <t xml:space="preserve">Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc1; final external publication remains.</t>
   </si>
   <si>
     <t xml:space="preserve">R-04</t>
@@ -1043,7 +1046,7 @@
     <t xml:space="preserve">Independent reviewer</t>
   </si>
   <si>
-    <t xml:space="preserve">Clean-clone replay at f22384acf925cebdd819915d17d530592d9ffba3 passed with exact PDF/HTML/figure hashes; independent reviewer confirmation and immutable tag remain.</t>
+    <t xml:space="preserve">Clean-clone replay at tagged v1.4.0-rc1 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
   </si>
   <si>
     <t xml:space="preserve">R-16</t>
@@ -1139,13 +1142,13 @@
     <t xml:space="preserve">Release tag</t>
   </si>
   <si>
-    <t xml:space="preserve">Pending immutable v1.4.0-rc1 tag; clean-clone replay verified at implementation candidate</t>
+    <t xml:space="preserve">v1.4.0-rc1 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
   </si>
   <si>
     <t xml:space="preserve">Publication manifest</t>
   </si>
   <si>
-    <t xml:space="preserve">publication_ready=false; local unrelated worktree changes; required test/artifact gates fresh; provider benchmark missing</t>
+    <t xml:space="preserve">publication_ready=false because provider benchmark/results are missing; clean-clone required test/artifact gates are fresh; shared local unrelated changes remain outside the candidate</t>
   </si>
   <si>
     <t xml:space="preserve">Required tests</t>
@@ -1181,7 +1184,7 @@
     <t xml:space="preserve">Manifest SHA-256</t>
   </si>
   <si>
-    <t xml:space="preserve">Pending final manifest regeneration after immutable tag</t>
+    <t xml:space="preserve">Manifest regenerated from the tagged clean clone; current hash is recorded in output/release_manifest.json</t>
   </si>
   <si>
     <t xml:space="preserve">Artifact</t>
@@ -2444,11 +2447,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="48742925"/>
-        <c:axId val="72750281"/>
+        <c:axId val="79066830"/>
+        <c:axId val="64259694"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="48742925"/>
+        <c:axId val="79066830"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2493,7 +2496,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72750281"/>
+        <c:crossAx val="64259694"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2501,7 +2504,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="72750281"/>
+        <c:axId val="64259694"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2546,7 +2549,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48742925"/>
+        <c:crossAx val="79066830"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2802,9 +2805,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>982440</xdr:colOff>
+      <xdr:colOff>982080</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>186120</xdr:rowOff>
+      <xdr:rowOff>185760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2813,7 +2816,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4299480" y="1609560"/>
-        <a:ext cx="4929840" cy="3424680"/>
+        <a:ext cx="4929480" cy="3424320"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4718,7 +4721,7 @@
         <v>249</v>
       </c>
       <c r="D20" s="41" t="s">
-        <v>135</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4729,7 +4732,7 @@
         <v>137</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D21" s="41" t="s">
         <v>141</v>
@@ -4743,7 +4746,7 @@
         <v>143</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D22" s="41" t="s">
         <v>147</v>
@@ -4757,7 +4760,7 @@
         <v>149</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D23" s="41" t="s">
         <v>153</v>
@@ -4771,7 +4774,7 @@
         <v>155</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D24" s="41" t="s">
         <v>159</v>
@@ -4785,7 +4788,7 @@
         <v>161</v>
       </c>
       <c r="C25" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D25" s="41" t="s">
         <v>165</v>
@@ -4799,7 +4802,7 @@
         <v>167</v>
       </c>
       <c r="C26" s="40" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D26" s="41" t="s">
         <v>171</v>
@@ -4813,7 +4816,7 @@
         <v>173</v>
       </c>
       <c r="C27" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D27" s="41" t="s">
         <v>176</v>
@@ -4827,7 +4830,7 @@
         <v>178</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D28" s="41" t="s">
         <v>181</v>
@@ -4841,7 +4844,7 @@
         <v>183</v>
       </c>
       <c r="C29" s="40" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D29" s="41" t="s">
         <v>187</v>
@@ -4855,7 +4858,7 @@
         <v>189</v>
       </c>
       <c r="C30" s="40" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D30" s="41" t="s">
         <v>192</v>
@@ -4869,7 +4872,7 @@
         <v>194</v>
       </c>
       <c r="C31" s="40" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D31" s="41" t="s">
         <v>198</v>
@@ -4883,7 +4886,7 @@
         <v>200</v>
       </c>
       <c r="C32" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D32" s="41" t="s">
         <v>204</v>
@@ -4897,7 +4900,7 @@
         <v>206</v>
       </c>
       <c r="C33" s="40" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D33" s="41" t="s">
         <v>209</v>
@@ -4911,7 +4914,7 @@
         <v>211</v>
       </c>
       <c r="C34" s="40" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D34" s="41" t="s">
         <v>214</v>
@@ -4925,7 +4928,7 @@
         <v>216</v>
       </c>
       <c r="C35" s="40" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D35" s="41" t="s">
         <v>220</v>
@@ -4967,7 +4970,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4977,7 +4980,7 @@
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4990,10 +4993,10 @@
         <v>33</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>38</v>
@@ -5002,18 +5005,18 @@
         <v>16</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="38" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B5" s="40" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D5" s="40" t="s">
         <v>134</v>
@@ -5022,38 +5025,38 @@
         <v>22</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="38" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D6" s="40" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E6" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="38" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D7" s="40" t="s">
         <v>134</v>
@@ -5062,347 +5065,347 @@
         <v>22</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D8" s="40" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E8" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="41" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D9" s="40" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E9" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="41" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D10" s="40" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E10" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="41" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C11" s="40" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E11" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F11" s="41" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C12" s="40" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E12" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F12" s="41" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="38" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B13" s="40" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E13" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="38" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B14" s="40" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C14" s="40" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E14" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F14" s="41" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="38" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D15" s="40" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E15" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="38" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C16" s="40" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D16" s="40" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E16" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F16" s="41" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="38" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D17" s="40" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E17" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="41" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="38" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C18" s="40" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D18" s="40" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E18" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F18" s="41" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="38" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C19" s="40" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D19" s="40" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E19" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F19" s="41" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="38" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C20" s="40" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D20" s="40" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="38" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D21" s="40" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E21" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F21" s="41" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="38" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B22" s="40" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D22" s="40" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E22" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F22" s="41" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="38" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B23" s="40" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D23" s="40" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E23" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F23" s="41" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="38" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D24" s="40" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E24" s="39" t="s">
         <v>18</v>
       </c>
       <c r="F24" s="41" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -5455,7 +5458,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="42" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -5463,172 +5466,172 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="43" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="43" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="43" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="45" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B15" s="45" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="45"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B16" s="46" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B17" s="46" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B18" s="46" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B19" s="46" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B20" s="46" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B21" s="46" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B22" s="46" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B23" s="46" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B24" s="46" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B25" s="46" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: finalize red-team evidence baseline
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc5 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc6 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc5; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc6; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc5; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc6; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc5; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc6; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc5 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc6 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc5 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc6 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc5 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc6 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc5 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc6 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc5; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc6; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc5 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc6 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc5 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc6 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc5 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc6 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc5 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc6 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: add causal gate mechanism contracts
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="409">
   <si>
     <t xml:space="preserve">Codomyrmex Review Action Register</t>
   </si>
@@ -449,7 +449,7 @@
     <t xml:space="preserve">Test maintainer</t>
   </si>
   <si>
-    <t xml:space="preserve">Exact locality, control, refusal, lifecycle, and mixed-severity contracts pass; broader mutation-sensitive mechanism tests for every named gate remain a release-review item.</t>
+    <t xml:space="preserve">Added seven real-component causal contracts covering budget, sandbox, trust tier/floor, risk pressure, completeness, recent-failure memory, and critical falsification. Each control/change pair asserts the expected score, decision, or diagnostic reason; the focused suite passes.</t>
   </si>
   <si>
     <t xml:space="preserve">A-018</t>
@@ -780,6 +780,9 @@
   </si>
   <si>
     <t xml:space="preserve">The critical/high FAILURE-pressure tests seed only three direct successes, yielding trust 0.22, which is below the separate 0.30 hard floor. REFUSE can therefore occur because of trust, and broad assertions such as HOLD-or-REFUSE do not prove the pressure mechanism.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seven real-component causal contracts cover every named gate mechanism with control/change pairs and exact score, decision, and reason assertions; the focused mutation-sensitive suite passes. Clean-clone replay remains part of the final verification.</t>
   </si>
   <si>
     <t xml:space="preserve">The gate uses maximum finding severity for its hard CRITICAL override; colony_falsify_plan averages finding weights and recommends execute below 0.4. A HIGH finding of weight 0.45 diluted by several LOW findings can receive an 'execute' recommendation even though the report verdict logic treats HIGH as FAIL.</t>
@@ -2447,11 +2450,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="79066830"/>
-        <c:axId val="64259694"/>
+        <c:axId val="97058062"/>
+        <c:axId val="87893316"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="79066830"/>
+        <c:axId val="97058062"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2496,7 +2499,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64259694"/>
+        <c:crossAx val="87893316"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2504,7 +2507,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64259694"/>
+        <c:axId val="87893316"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2549,7 +2552,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79066830"/>
+        <c:crossAx val="97058062"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2805,9 +2808,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>982080</xdr:colOff>
+      <xdr:colOff>981720</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>185760</xdr:rowOff>
+      <xdr:rowOff>185400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2816,7 +2819,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4299480" y="1609560"/>
-        <a:ext cx="4929480" cy="3424320"/>
+        <a:ext cx="4929120" cy="3423960"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3252,7 +3255,7 @@
       </c>
       <c r="B19" s="29" t="n">
         <f aca="false">COUNTIF('Action Register'!$H$5:$H$35,A19)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" s="30" t="s">
         <v>21</v>
@@ -3264,7 +3267,7 @@
       </c>
       <c r="B20" s="29" t="n">
         <f aca="false">COUNTIF('Action Register'!$H$5:$H$35,A20)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C20" s="30" t="s">
         <v>23</v>
@@ -3988,7 +3991,7 @@
         <v>140</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I21" s="41" t="s">
         <v>141</v>
@@ -4735,7 +4738,7 @@
         <v>251</v>
       </c>
       <c r="D21" s="41" t="s">
-        <v>141</v>
+        <v>252</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4746,7 +4749,7 @@
         <v>143</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D22" s="41" t="s">
         <v>147</v>
@@ -4760,7 +4763,7 @@
         <v>149</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D23" s="41" t="s">
         <v>153</v>
@@ -4774,7 +4777,7 @@
         <v>155</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D24" s="41" t="s">
         <v>159</v>
@@ -4788,7 +4791,7 @@
         <v>161</v>
       </c>
       <c r="C25" s="40" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D25" s="41" t="s">
         <v>165</v>
@@ -4802,7 +4805,7 @@
         <v>167</v>
       </c>
       <c r="C26" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D26" s="41" t="s">
         <v>171</v>
@@ -4816,7 +4819,7 @@
         <v>173</v>
       </c>
       <c r="C27" s="40" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D27" s="41" t="s">
         <v>176</v>
@@ -4830,7 +4833,7 @@
         <v>178</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D28" s="41" t="s">
         <v>181</v>
@@ -4844,7 +4847,7 @@
         <v>183</v>
       </c>
       <c r="C29" s="40" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D29" s="41" t="s">
         <v>187</v>
@@ -4858,7 +4861,7 @@
         <v>189</v>
       </c>
       <c r="C30" s="40" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D30" s="41" t="s">
         <v>192</v>
@@ -4872,7 +4875,7 @@
         <v>194</v>
       </c>
       <c r="C31" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D31" s="41" t="s">
         <v>198</v>
@@ -4886,7 +4889,7 @@
         <v>200</v>
       </c>
       <c r="C32" s="40" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D32" s="41" t="s">
         <v>204</v>
@@ -4900,7 +4903,7 @@
         <v>206</v>
       </c>
       <c r="C33" s="40" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D33" s="41" t="s">
         <v>209</v>
@@ -4914,7 +4917,7 @@
         <v>211</v>
       </c>
       <c r="C34" s="40" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D34" s="41" t="s">
         <v>214</v>
@@ -4928,7 +4931,7 @@
         <v>216</v>
       </c>
       <c r="C35" s="40" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D35" s="41" t="s">
         <v>220</v>
@@ -4970,7 +4973,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4980,7 +4983,7 @@
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4993,10 +4996,10 @@
         <v>33</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>38</v>
@@ -5005,18 +5008,18 @@
         <v>16</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="38" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B5" s="40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D5" s="40" t="s">
         <v>134</v>
@@ -5025,38 +5028,38 @@
         <v>22</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="38" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D6" s="40" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E6" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="38" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D7" s="40" t="s">
         <v>134</v>
@@ -5065,347 +5068,347 @@
         <v>22</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D8" s="40" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E8" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="41" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D9" s="40" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E9" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="41" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D10" s="40" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E10" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="41" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C11" s="40" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E11" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F11" s="41" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C12" s="40" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E12" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F12" s="41" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="38" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B13" s="40" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E13" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="38" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B14" s="40" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C14" s="40" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E14" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F14" s="41" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="38" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D15" s="40" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E15" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="38" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C16" s="40" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D16" s="40" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E16" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F16" s="41" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="38" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D17" s="40" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E17" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="41" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="38" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C18" s="40" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D18" s="40" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E18" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F18" s="41" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="38" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C19" s="40" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D19" s="40" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E19" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F19" s="41" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="38" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C20" s="40" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D20" s="40" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="38" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D21" s="40" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E21" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F21" s="41" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="38" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B22" s="40" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D22" s="40" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E22" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F22" s="41" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="38" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B23" s="40" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D23" s="40" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E23" s="39" t="s">
         <v>22</v>
       </c>
       <c r="F23" s="41" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="38" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C24" s="40" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D24" s="40" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E24" s="39" t="s">
         <v>18</v>
       </c>
       <c r="F24" s="41" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -5458,7 +5461,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="42" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -5466,172 +5469,172 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="43" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="43" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="43" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="45" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B15" s="45" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C15" s="45"/>
       <c r="D15" s="45"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B16" s="46" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B17" s="46" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B18" s="46" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B19" s="46" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B20" s="46" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B21" s="46" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B22" s="46" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B23" s="46" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B24" s="46" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B25" s="46" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: seal publication evidence candidate
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Codomyrmex Review Action Register</t>
   </si>
   <si>
-    <t xml:space="preserve">Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Implementation candidate 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025 | Evidence 14 July 2026</t>
+    <t xml:space="preserve">Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Implementation candidate f22384acf925cebdd819915d17d530592d9ffba3 | Evidence 14 July 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Open blockers</t>
@@ -200,7 +200,7 @@
     <t xml:space="preserve">Daniel + test/release maintainer</t>
   </si>
   <si>
-    <t xml:space="preserve">Fresh candidate run: 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; branch 74.10714285714286% (581/784); line 82.44274809160305% (2,227/2,622); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone verification remains.</t>
+    <t xml:space="preserve">Fresh candidate run: 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; branch 74.29667519181585% (581/782); line 82.57419923596827% (2,229/2,621); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone verification remains.</t>
   </si>
   <si>
     <t xml:space="preserve">A-004</t>
@@ -431,7 +431,7 @@
     <t xml:space="preserve">Release maintainer</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidate evidence exists with PDF SHA-256 2f6f10e2cac4ac357003cc278a86242806a660e6167dcb95da71983b2993c6e8, manifest SHA-256 f1816c40725f035019d85041ba350a54324e83cc37adc1b2f54f3d3df595a60f, JUnit, coverage, variables, figures, and expanded manuscript; immutable release/tag attachment remains open.</t>
+    <t xml:space="preserve">Candidate evidence exists with PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2, manifest SHA-256 manifest pending final immutable-release verification, JUnit, coverage, variables, figures, and expanded manuscript; immutable release/tag attachment remains open.</t>
   </si>
   <si>
     <t xml:space="preserve">A-017</t>
@@ -701,7 +701,7 @@
     <t xml:space="preserve">Evidence summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Current candidate evidence (1db2b7a326b4)</t>
+    <t xml:space="preserve">Current candidate evidence (f22384acf925)</t>
   </si>
   <si>
     <t xml:space="preserve">Attached PDF: 50 pages, SHA-256 c1432347b75c34258fb53d29b4d747684fbc06655126fd5af37182b0928a4270. Public main at e85aee6758726ca1fbba202d0ef1a09d524029e3 contains a 77-page output/paper.pdf, SHA-256 6333fde6bd65aa25406ce5491424010ec5b15f932093e3ea64954d91f0a7723d. Public 02_methodology.md says FAILURE does not directly reduce risk_ok, while the attachment says max(RISK, FAILURE); the public abstract also retains stronger persistence/control claims.</t>
@@ -716,7 +716,7 @@
     <t xml:space="preserve">Attachment reports 773 passing tests and 78.7% branch coverage. Public main produced 764 collected, 763 passed, 1 skipped, and 475/606 branches covered = 78.382838...%, reported as 78.4%. Ruff and ty both reproduced at zero.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fresh candidate run: 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; branch 74.10714285714286% (581/784); line 82.44274809160305% (2,227/2,622); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+    <t xml:space="preserve">Fresh candidate run: 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; branch 74.29667519181585% (581/782); line 82.57419923596827% (2,229/2,621); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
   </si>
   <si>
     <t xml:space="preserve">The attachment instructs ./run.sh --pipeline --project ongoing/codomyrmex --core-only and then cd projects/ongoing/codomyrmex. Public main contains neither run.sh nor projects/ongoing/codomyrmex.</t>
@@ -845,7 +845,7 @@
     <t xml:space="preserve">Full Git SHA, clean status, dependency lock hash, config digest and source archive are recorded.</t>
   </si>
   <si>
-    <t xml:space="preserve">Manifest candidate records implementation revision 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025, lock/config/source hashes, tools, status, and artifact hashes; local unrelated changes remain outside the candidate; immutable tag pending.</t>
+    <t xml:space="preserve">Manifest candidate records implementation revision f22384acf925cebdd819915d17d530592d9ffba3, lock/config/source hashes, tools, status, and artifact hashes; local unrelated changes remain outside the candidate; immutable tag pending.</t>
   </si>
   <si>
     <t xml:space="preserve">R-02</t>
@@ -860,7 +860,7 @@
     <t xml:space="preserve">Manuscript/release</t>
   </si>
   <si>
-    <t xml:space="preserve">Canonical PDF SHA-256 36ebc8982f92d5bd007b92f9415d029dfc26ee4c5aa185c0345fc8b48b1f0f76; clean clone at 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025 regenerated the exact PDF, HTML, and figure hashes with SOURCE_DATE_EPOCH pinning; immutable tag pending.</t>
+    <t xml:space="preserve">Canonical PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2; clean clone at f22384acf925cebdd819915d17d530592d9ffba3 regenerated the exact PDF, HTML, and figure hashes with SOURCE_DATE_EPOCH pinning; immutable tag pending.</t>
   </si>
   <si>
     <t xml:space="preserve">R-03</t>
@@ -872,7 +872,7 @@
     <t xml:space="preserve">The manuscript, source, tests, generated variables and rendered artifacts all come from the same tagged revision.</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidate source, variables, coverage, JUnit, HTML, PDF, and figures were regenerated at 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025; clean-clone hashes match; immutable tag pending.</t>
+    <t xml:space="preserve">Candidate source, variables, coverage, JUnit, HTML, PDF, and figures were regenerated at f22384acf925cebdd819915d17d530592d9ffba3; clean-clone hashes match; immutable tag pending.</t>
   </si>
   <si>
     <t xml:space="preserve">R-04</t>
@@ -1043,7 +1043,7 @@
     <t xml:space="preserve">Independent reviewer</t>
   </si>
   <si>
-    <t xml:space="preserve">Clean-clone replay at 1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025 passed with exact PDF/HTML/figure hashes; independent reviewer confirmation and immutable tag remain.</t>
+    <t xml:space="preserve">Clean-clone replay at f22384acf925cebdd819915d17d530592d9ffba3 passed with exact PDF/HTML/figure hashes; independent reviewer confirmation and immutable tag remain.</t>
   </si>
   <si>
     <t xml:space="preserve">R-16</t>
@@ -1133,7 +1133,7 @@
     <t xml:space="preserve">Current evaluated revision</t>
   </si>
   <si>
-    <t xml:space="preserve">1db2b7a326b468a6c33ce9af7adb8e2ddd5d8025</t>
+    <t xml:space="preserve">f22384acf925cebdd819915d17d530592d9ffba3</t>
   </si>
   <si>
     <t xml:space="preserve">Release tag</t>
@@ -1175,7 +1175,7 @@
     <t xml:space="preserve">Canonical PDF SHA-256</t>
   </si>
   <si>
-    <t xml:space="preserve">36ebc8982f92d5bd007b92f9415d029dfc26ee4c5aa185c0345fc8b48b1f0f76</t>
+    <t xml:space="preserve">4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2</t>
   </si>
   <si>
     <t xml:space="preserve">Manifest SHA-256</t>
@@ -1196,37 +1196,37 @@
     <t xml:space="preserve">output/paper.html</t>
   </si>
   <si>
-    <t xml:space="preserve">6d999977449e85e979992f07c16472bdea07e5ab8e8018ce34a421e0938120df</t>
+    <t xml:space="preserve">7b1f10d08475204af555e798de31c13158c9a7112586717c7aba906230cd1200</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/manuscript_variables.json</t>
   </si>
   <si>
-    <t xml:space="preserve">6b424188e10d340dce60cb520809ab30ab3014fb9681b7935befa63271b86c98</t>
+    <t xml:space="preserve">3fc5e6ef13443a1a214722f24332b8db0fcd3fbce3c3bcda69af7dbb43e080de</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_coverage.json</t>
   </si>
   <si>
-    <t xml:space="preserve">117dcb7145d1455a2f0125e954c92ff016012622e7e1f6a951b26996541cceb2</t>
+    <t xml:space="preserve">e5f1b3ac69ebeda28cded7cd28ed5a9c2e03c7a772222857a08143a7dc37b2b6</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_test_report.xml</t>
   </si>
   <si>
-    <t xml:space="preserve">0dad5f0f470c4bf770bf7bb3f15169099113e4e28a8f6af203caf232c7102355</t>
+    <t xml:space="preserve">832bc840a1c36264c34e7169e9b7e3bff58b41b6c58ff6e09aff4dcce31dceba</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_test_status.json</t>
   </si>
   <si>
-    <t xml:space="preserve">abe20b74d40742d444770bc68e96979f916c8766971eaca62759d01ee12657af</t>
+    <t xml:space="preserve">88e9076c9961a314a2394dff21917b9ccbd490c9bcbabca7ea4c41b4d4efdf35</t>
   </si>
   <si>
     <t xml:space="preserve">output/release_manifest.json</t>
   </si>
   <si>
-    <t xml:space="preserve">4128b0a0fec2bd036cab9f2b12d19b010b6614efe190fea3640aa1fb2d946a3f</t>
+    <t xml:space="preserve">Pending final manifest regeneration after immutable release-candidate tag</t>
   </si>
   <si>
     <t xml:space="preserve">Enforcement profile</t>
@@ -2444,11 +2444,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="75438293"/>
-        <c:axId val="54312665"/>
+        <c:axId val="48742925"/>
+        <c:axId val="72750281"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="75438293"/>
+        <c:axId val="48742925"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2493,7 +2493,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54312665"/>
+        <c:crossAx val="72750281"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2501,7 +2501,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="54312665"/>
+        <c:axId val="72750281"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2546,7 +2546,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75438293"/>
+        <c:crossAx val="48742925"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2802,9 +2802,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>983160</xdr:colOff>
+      <xdr:colOff>982440</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>186840</xdr:rowOff>
+      <xdr:rowOff>186120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2813,7 +2813,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4299480" y="1609560"/>
-        <a:ext cx="4930560" cy="3425400"/>
+        <a:ext cx="4929840" cy="3424680"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">

</xml_diff>

<commit_message>
docs: align coverage gate and release register
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,10 +2065,11 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc4 (full revision recorded in manifest) | Evidence 14 July 2026</t>
-        </is>
-      </c>
-    </row>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc5 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="48">
       <c r="A4" s="51" t="inlineStr">
         <is>
@@ -2130,6 +2131,7 @@
       <c r="H6" s="76" t="n"/>
       <c r="I6" s="77" t="n"/>
     </row>
+    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="48">
       <c r="A8" s="78" t="inlineStr">
         <is>
@@ -2229,6 +2231,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="48">
       <c r="A16" s="78" t="inlineStr">
         <is>
@@ -2333,6 +2336,8 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25" ht="15" customHeight="1" s="48">
       <c r="A25" s="100" t="inlineStr">
         <is>
@@ -2370,6 +2375,7 @@
       <c r="H28" s="107" t="n"/>
       <c r="I28" s="108" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="48">
       <c r="A30" s="109" t="inlineStr">
         <is>
@@ -2471,6 +2477,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="48">
       <c r="A4" s="79" t="inlineStr">
         <is>
@@ -2514,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc4; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc5; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc4; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc5; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -4058,6 +4065,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="48">
       <c r="A4" s="79" t="inlineStr">
         <is>
@@ -4098,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc4; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc5; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc4 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc5 is complete.</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4208,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4274,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc4 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc5 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4807,6 +4815,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="48">
       <c r="A4" s="79" t="inlineStr">
         <is>
@@ -4867,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc4 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc5 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc4 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc5 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc4 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc5 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc4; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc5; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5315,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc4 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc5 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc4 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc5 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc4 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc5 also passes.</t>
         </is>
       </c>
     </row>
@@ -5531,6 +5540,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="48">
       <c r="A3" s="116" t="inlineStr">
         <is>
@@ -5563,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc4 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc5 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>
@@ -5651,6 +5661,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
test: close gate mechanism evidence gap
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -200,7 +200,7 @@
     <t xml:space="preserve">Daniel + test/release maintainer</t>
   </si>
   <si>
-    <t xml:space="preserve">Fresh candidate run: 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; branch 74.29667519181585% (581/782); line 82.57419923596827% (2,229/2,621); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone verification remains.</t>
+    <t xml:space="preserve">Fresh candidate run: 822 collected / 822 passed / 0 skipped / 0 failed / 0 errors; branch 74.29667519181585% (581/782); line 82.57419923596827% (2,229/2,621); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone verification remains.</t>
   </si>
   <si>
     <t xml:space="preserve">A-004</t>
@@ -431,7 +431,7 @@
     <t xml:space="preserve">Release maintainer</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidate evidence exists with PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2, manifest SHA-256 manifest pending final immutable-release verification, JUnit, coverage, variables, figures, and expanded manuscript; immutable release/tag attachment remains open.</t>
+    <t xml:space="preserve">Candidate evidence exists with PDF SHA-256 37bc6ba55b8208a8a455c8e82371b848a5378c82b5a6d0f72ce43a1ee58894bd, manifest SHA-256 manifest pending final immutable-release verification, JUnit, coverage, variables, figures, and expanded manuscript; immutable release/tag attachment remains open.</t>
   </si>
   <si>
     <t xml:space="preserve">A-017</t>
@@ -716,7 +716,7 @@
     <t xml:space="preserve">Attachment reports 773 passing tests and 78.7% branch coverage. Public main produced 764 collected, 763 passed, 1 skipped, and 475/606 branches covered = 78.382838...%, reported as 78.4%. Ruff and ty both reproduced at zero.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fresh candidate run: 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; branch 74.29667519181585% (581/782); line 82.57419923596827% (2,229/2,621); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+    <t xml:space="preserve">Fresh candidate run: 822 collected / 822 passed / 0 skipped / 0 failed / 0 errors; branch 74.29667519181585% (581/782); line 82.57419923596827% (2,229/2,621); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at the implementation candidate regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
   </si>
   <si>
     <t xml:space="preserve">The attachment instructs ./run.sh --pipeline --project ongoing/codomyrmex --core-only and then cd projects/ongoing/codomyrmex. Public main contains neither run.sh nor projects/ongoing/codomyrmex.</t>
@@ -776,7 +776,7 @@
     <t xml:space="preserve">git ls-files output lists only output/paper.html and output/paper.pdf. Generated manuscript_variables.json, colony_kernel_coverage.json and expanded manuscript files are ignored. figure_registry.json and output/figures were absent in the audit checkout.</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidate evidence and the clean-clone release package exist with PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
+    <t xml:space="preserve">Candidate evidence and the clean-clone release package exist with PDF SHA-256 37bc6ba55b8208a8a455c8e82371b848a5378c82b5a6d0f72ce43a1ee58894bd, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
   </si>
   <si>
     <t xml:space="preserve">The critical/high FAILURE-pressure tests seed only three direct successes, yielding trust 0.22, which is below the separate 0.30 hard floor. REFUSE can therefore occur because of trust, and broad assertions such as HOLD-or-REFUSE do not prove the pressure mechanism.</t>
@@ -866,7 +866,7 @@
     <t xml:space="preserve">Manuscript/release</t>
   </si>
   <si>
-    <t xml:space="preserve">Canonical PDF SHA-256 4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2; clean clone at tagged v1.4.0-rc1 regenerated the exact PDF, HTML, evidence, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+    <t xml:space="preserve">Canonical PDF SHA-256 37bc6ba55b8208a8a455c8e82371b848a5378c82b5a6d0f72ce43a1ee58894bd; clean clone at tagged v1.4.0-rc1 regenerated the exact PDF, HTML, evidence, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
   </si>
   <si>
     <t xml:space="preserve">R-03</t>
@@ -1004,7 +1004,7 @@
     <t xml:space="preserve">Test/release</t>
   </si>
   <si>
-    <t xml:space="preserve">Machine status reports 815 collected / 815 passed / 0 skipped / 0 failed / 0 errors; coverage reports exact numerators/denominators.</t>
+    <t xml:space="preserve">Machine status reports 822 collected / 822 passed / 0 skipped / 0 failed / 0 errors; coverage reports exact numerators/denominators.</t>
   </si>
   <si>
     <t xml:space="preserve">R-13</t>
@@ -1157,7 +1157,7 @@
     <t xml:space="preserve">Required tests</t>
   </si>
   <si>
-    <t xml:space="preserve">815 collected / 815 passed / 0 skipped / 0 failed / 0 errors</t>
+    <t xml:space="preserve">822 collected / 822 passed / 0 skipped / 0 failed / 0 errors</t>
   </si>
   <si>
     <t xml:space="preserve">Coverage</t>
@@ -1181,7 +1181,7 @@
     <t xml:space="preserve">Canonical PDF SHA-256</t>
   </si>
   <si>
-    <t xml:space="preserve">4de816030843c5d43255dfb6a8d0a8056091689ad6d667d08d6569a5529f92c2</t>
+    <t xml:space="preserve">37bc6ba55b8208a8a455c8e82371b848a5378c82b5a6d0f72ce43a1ee58894bd</t>
   </si>
   <si>
     <t xml:space="preserve">Manifest SHA-256</t>
@@ -1202,13 +1202,13 @@
     <t xml:space="preserve">output/paper.html</t>
   </si>
   <si>
-    <t xml:space="preserve">7b1f10d08475204af555e798de31c13158c9a7112586717c7aba906230cd1200</t>
+    <t xml:space="preserve">f930564711c845f6e6abc494ed81a463202efce466929ea23a83d85110151df3</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/manuscript_variables.json</t>
   </si>
   <si>
-    <t xml:space="preserve">3fc5e6ef13443a1a214722f24332b8db0fcd3fbce3c3bcda69af7dbb43e080de</t>
+    <t xml:space="preserve">2445b34cdaa162b0ee27ae050316b42e7ba09e2a5ecf4b09623f443f3a28e52d</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_coverage.json</t>
@@ -1220,13 +1220,13 @@
     <t xml:space="preserve">output/data/colony_kernel_test_report.xml</t>
   </si>
   <si>
-    <t xml:space="preserve">832bc840a1c36264c34e7169e9b7e3bff58b41b6c58ff6e09aff4dcce31dceba</t>
+    <t xml:space="preserve">59498b92044f4082c05d1a60fdb482ea9efe4fb761e79db0d4a7077f5fb7694f</t>
   </si>
   <si>
     <t xml:space="preserve">output/data/colony_kernel_test_status.json</t>
   </si>
   <si>
-    <t xml:space="preserve">88e9076c9961a314a2394dff21917b9ccbd490c9bcbabca7ea4c41b4d4efdf35</t>
+    <t xml:space="preserve">ad5ee65f8e1933d05928cf59a555c56f48cb0a47510972b8d0006ecd09bc9d19</t>
   </si>
   <si>
     <t xml:space="preserve">output/release_manifest.json</t>
@@ -2450,11 +2450,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97058062"/>
-        <c:axId val="87893316"/>
+        <c:axId val="27935626"/>
+        <c:axId val="60479080"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97058062"/>
+        <c:axId val="27935626"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2499,7 +2499,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87893316"/>
+        <c:crossAx val="60479080"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2507,7 +2507,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87893316"/>
+        <c:axId val="60479080"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2552,7 +2552,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97058062"/>
+        <c:crossAx val="27935626"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2808,9 +2808,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>981720</xdr:colOff>
+      <xdr:colOff>981360</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>185400</xdr:rowOff>
+      <xdr:rowOff>185040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2819,7 +2819,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4299480" y="1609560"/>
-        <a:ext cx="4929120" cy="3423960"/>
+        <a:ext cx="4928760" cy="3423600"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">

</xml_diff>

<commit_message>
docs: synchronize rc8 publication evidence
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc6 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc8 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc6; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc8; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc6; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc8; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc6; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc8; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc6 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc8 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc6 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc6 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc8 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc6 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc8 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc6 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc8 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc6; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc8; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc6 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc8 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc6 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc8 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc6 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc8 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc6 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc8 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release: pin regenerated html artifact
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc8 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc9 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc8; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc9; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc8; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc9; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc8; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc9; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc8 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc9 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc8 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc8 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc9 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc8 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc9 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc8 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc9 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc8; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc9; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc8 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc9 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc8 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc9 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc8 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc9 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc8 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc9 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: finalize rc11 evidence hashes
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc10 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc11 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc10; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc11; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc10; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc11; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc10; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc11; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc10 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc11 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc10 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc11 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc10 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc11 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc10 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc11 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc10; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc11; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc10 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc11 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc10 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc11 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc10 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc11 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc10 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc11 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release: pin reproducible rc10 artifacts
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc9 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc10 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc9; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc10; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc9; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc10; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc9; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc10; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc9 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc10 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc9 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc10 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc9 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc10 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc9 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc10 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc9 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc10 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc9; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc10; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc9 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc10 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc9 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc10 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc9 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc10 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc9 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc10 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release: harden benchmark evidence and manuscript boundaries
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc11 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc12 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc11; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc12; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc11; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc12; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Fresh candidate run: 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="I18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 826/826 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 833/833 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc11; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc12; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc11 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc12 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc11 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="D18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 826/826 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 833/833 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="D20" s="114" t="inlineStr">
         <is>
-          <t>Candidate evidence and the clean-clone release package exist with PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
+          <t>Candidate evidence and the clean-clone release package exist with PDF SHA-256 9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc11 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc12 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc11 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc12 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706; clean clone at tagged v1.4.0-rc11 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75; clean clone at tagged v1.4.0-rc12 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc11; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc12; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5228,7 @@
       </c>
       <c r="F16" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="F17" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors; pytest collected 827 items and deselected 1; coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors; pytest collected 834 items and deselected 1; coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc11 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc12 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc11 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc12 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc11 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc12 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc11 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc12 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="B7" s="117" t="inlineStr">
         <is>
-          <t>826 JUnit-collected / 826 passed / 0 skipped / 0 failed / 0 errors (827 pytest items collected; 1 deselected)</t>
+          <t>833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected)</t>
         </is>
       </c>
     </row>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="B11" s="117" t="inlineStr">
         <is>
-          <t>69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706</t>
+          <t>9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75</t>
         </is>
       </c>
     </row>
@@ -5670,7 +5670,7 @@
       </c>
       <c r="B14" s="47" t="inlineStr">
         <is>
-          <t>69fdbb018d81b7b5dd0ae170187842ef30647b8f6864af91f615fa23ea6ac706</t>
+          <t>9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B15" s="118" t="inlineStr">
         <is>
-          <t>cb0f7bd1546dc8acca60dccc355e4093ad1a2bd7e9f878dad7a9413e2b0641f5</t>
+          <t>ec6dcff2a8b4035c63530479b0af279dcd5e5bb79acc22a65df68d50dd4386e2</t>
         </is>
       </c>
       <c r="C15" s="118" t="n"/>
@@ -5696,7 +5696,7 @@
       </c>
       <c r="B16" s="119" t="inlineStr">
         <is>
-          <t>865ba48c143b1b5fbfb98a79cf94638b673d0ec208acc68a95857d64410</t>
+          <t>ab097f586bc3039830962988eb9df8ecf64c40d1dcdca0112958e53c9d7e13db</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="B17" s="119" t="inlineStr">
         <is>
-          <t>7dc284a8b6d29c163eb2185e1372795dfb3da8eb22977c66a289286249239ccf</t>
+          <t>abd7dae63df1a6be3e0e4bd3d5c1423d598ac39ea71853bfa6abad69abf23f6b</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="B18" s="119" t="inlineStr">
         <is>
-          <t>677e30d935cc5e09849d92e9d6ea3c014d8d8ee076aaa5dd8573d9cc7002a1ce</t>
+          <t>6c442af40d8005c6bad25b690107a9548252bf96dca621c75b5075a362c9a778</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
       </c>
       <c r="B19" s="119" t="inlineStr">
         <is>
-          <t>53be36e539e2e45ea55b78758280cb9e5a1e81f30968619a326618123b070dbf</t>
+          <t>859a674b509ae72973ac10b78b5a9c7ef6a6118e4128c16695495781f9910b25</t>
         </is>
       </c>
     </row>
@@ -5756,7 +5756,7 @@
       </c>
       <c r="B21" s="119" t="inlineStr">
         <is>
-          <t>ad5ee65f8e1933d05928cf59a555c56f48cb0a47510972b8d0006ecd09bc9d19</t>
+          <t>859a674b509ae72973ac10b78b5a9c7ef6a6118e4128c16695495781f9910b25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release: harden benchmark receipt provenance
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc12 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc13 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc12; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc13; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc12; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc13; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Fresh candidate run: 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="I18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 833/833 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 841/841 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc12; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc13; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc12 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc12 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="D18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 833/833 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 841/841 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc12 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc13 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc12 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc13 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75; clean clone at tagged v1.4.0-rc12 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75; clean clone at tagged v1.4.0-rc13 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc12; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc13; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5228,7 @@
       </c>
       <c r="F16" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="F17" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors; pytest collected 834 items and deselected 1; coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors; pytest collected 842 items and deselected 1; coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc12 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc13 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc12 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc13 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc12 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc13 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc12 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc13 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="B7" s="117" t="inlineStr">
         <is>
-          <t>833 JUnit-collected / 833 passed / 0 skipped / 0 failed / 0 errors (834 pytest items collected; 1 deselected)</t>
+          <t>841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: pin rc13 evidence snapshot
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc13 is complete.</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="I18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 841/841 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 840/840 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="D18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 841/841 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 840/840 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="D20" s="114" t="inlineStr">
         <is>
-          <t>Candidate evidence and the clean-clone release package exist with PDF SHA-256 9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
+          <t>Candidate evidence and the clean-clone release package exist with PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75; clean clone at tagged v1.4.0-rc13 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc13 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5228,7 @@
       </c>
       <c r="F16" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="F17" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors; pytest collected 842 items and deselected 1; coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors; pytest collected 841 items and deselected 1; coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="B7" s="117" t="inlineStr">
         <is>
-          <t>841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (842 pytest items collected; 1 deselected)</t>
+          <t>840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected)</t>
         </is>
       </c>
     </row>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="B11" s="117" t="inlineStr">
         <is>
-          <t>9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75</t>
+          <t>3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d</t>
         </is>
       </c>
     </row>
@@ -5670,7 +5670,7 @@
       </c>
       <c r="B14" s="47" t="inlineStr">
         <is>
-          <t>9a463ff0f52a254115920206a677104423658f3fcb359f6b00e620c70aae9a75</t>
+          <t>3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B15" s="118" t="inlineStr">
         <is>
-          <t>ec6dcff2a8b4035c63530479b0af279dcd5e5bb79acc22a65df68d50dd4386e2</t>
+          <t>7f42c41a1f42127cf9b06ebc5a53384ecaa5a57fd51a7e2feb84cc0b29999355</t>
         </is>
       </c>
       <c r="C15" s="118" t="n"/>
@@ -5696,7 +5696,7 @@
       </c>
       <c r="B16" s="119" t="inlineStr">
         <is>
-          <t>ab097f586bc3039830962988eb9df8ecf64c40d1dcdca0112958e53c9d7e13db</t>
+          <t>49ba171b55cd8946d1024dbcbbca12fbe1986e90d3ed152d695c1501f1b44e85</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="B17" s="119" t="inlineStr">
         <is>
-          <t>abd7dae63df1a6be3e0e4bd3d5c1423d598ac39ea71853bfa6abad69abf23f6b</t>
+          <t>e7134083deb0d91cb91bfed463ae7809d3d461d22a067c85ac84fe740d004e57</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="B18" s="119" t="inlineStr">
         <is>
-          <t>6c442af40d8005c6bad25b690107a9548252bf96dca621c75b5075a362c9a778</t>
+          <t>cbcfc215fee2cf2200ee0c1ae18e2adf5a2ec9d58c360ef8e691b0b5be963e5eb</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
       </c>
       <c r="B19" s="119" t="inlineStr">
         <is>
-          <t>859a674b509ae72973ac10b78b5a9c7ef6a6118e4128c16695495781f9910b25</t>
+          <t>fc2f174b03c69d8d3bf038e6e49c11b1c86d39aa74920aa7c226211e6e4a1ecf</t>
         </is>
       </c>
     </row>
@@ -5756,7 +5756,7 @@
       </c>
       <c r="B21" s="119" t="inlineStr">
         <is>
-          <t>859a674b509ae72973ac10b78b5a9c7ef6a6118e4128c16695495781f9910b25</t>
+          <t>fc2f174b03c69d8d3bf038e6e49c11b1c86d39aa74920aa7c226211e6e4a1ecf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: correct rc14 provenance references
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc13 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc14 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc13; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc14; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc13; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc14; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc13; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc14; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc13 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc14 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc13 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc13 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc14 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc13 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc14 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc13 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc14 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc13; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc14; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc13 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc14 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc13 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc14 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc13 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc14 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc13 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc14 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: isolate authorization expiry timing
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc14 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc15 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc14; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc15; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc14; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc15; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc14; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc15; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc14 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc15 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc14 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc14 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc15 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc14 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc15 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc14 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc15 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc14; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc15; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc14 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc15 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc14 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc15 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc14 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc15 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc14 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc15 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: advance candidate provenance to rc16
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc15 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc16 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc15; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc16; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc15; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc16; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc15; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc16; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc15 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc16 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc15 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc15 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc16 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc15 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc16 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc15 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc16 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc15; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc16; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc15 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc16 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc15 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc16 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc15 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc16 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc15 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc16 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: pin final candidate provenance
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc16 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc18 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc16; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc18; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc16; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc18; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc16; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc18; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc16 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc18 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc16 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc16 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc18 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc16 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc18 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc16 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc18 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc16; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc18; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc16 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc18 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc16 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc18 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc16 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc18 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc16 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc18 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: correct final candidate audit label
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc18 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc19 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc18; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc19; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc18; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc19; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc18; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc19; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc18 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc19 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc18 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc18 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc19 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc18 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc19 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc18 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc19 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc18; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc19; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc18 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc19 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc18 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc19 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc18 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc19 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc18 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc19 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: advance publication candidate to rc20
</commit_message>
<xml_diff>
--- a/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
+++ b/review_artifacts/Codomyrmex_Action_Register_2026-07-13_Follow_Up.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2" ht="21.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc19 (full revision recorded in manifest) | Evidence 14 July 2026</t>
+          <t>Consolidated first- and second-pass review | Historical audit e85aee6758726ca1fbba202d0ef1a09d524029e3 | Follow-up baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837 | Publication candidate v1.4.0-rc20 (full revision recorded in manifest) | Evidence 14 July 2026</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I4" s="110" t="inlineStr">
         <is>
-          <t>Current candidate follow-up (v1.4.0-rc19; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
+          <t>Current candidate follow-up (v1.4.0-rc20; baseline 4bd6c1804f2caa905d36bcb39d67bdf8c1d86837)</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc19; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc20; clean-clone verifier passes all available integrity gates. Publication remains held by R-20 and public evidence attachment.</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Fresh candidate run: 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="I8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="I9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="I10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="I13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="I18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 840/840 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 841/841 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Candidate is committed and tagged v1.4.0-rc19; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
+          <t>Candidate is committed and tagged v1.4.0-rc20; the clean-clone replay and manifest pass all available gates. v1.4.0 publication and external evidence attachment remain required.</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Implemented and tested from real kernel components: 0.875 EXECUTE -&gt; 0.725 HOLD at same target after TEST FAILURE pressure 3.0; unrelated target and 20-tick recovery return 0.875 EXECUTE. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Fresh candidate run: 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Fresh candidate run: 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); branch 74.37185929648241% (592/796 branches); line 82.59604190919674% (2,246/2,640 lines); floor 60.0%. Machine-readable status/JUnit/coverage are current. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc19 is complete.</t>
+          <t>Reproduction commands operate from the Codomyrmex root and use the local compiler/generator. Clean-clone replay at v1.4.0-rc20 is complete.</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ColonyKernel shares ConsequenceMemory with ActuationGate; causal locality and trust-pressure contracts pass in the publication suite. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Real ResourceLedger contracts cover all seven dimensions; standalone over-budget is REFUSE/0.0 and integrated routing is documented HOLD. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="D11" s="114" t="inlineStr">
         <is>
-          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>ActionProposal has one typed conversion to the complete falsification plan; every named field is covered by production-component tests. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict profile now requires signed, scoped, expiring, single-use authorization plus executor receipt; unattested reports are quarantined and cannot mutate trust/failure state. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Strict RegisteredActionExecutor rejects direct protected execution without a consumed authorization; advisory mode remains explicitly bypassable. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc19 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
+          <t>Governed action scope is explicit for patch_file, run_tests, and archive_module; absolute/traversal/out-of-scope targets fail closed. Clean-clone replay at tagged v1.4.0-rc20 regenerated matching PDF, HTML, and figure hashes; immutable tag and provider benchmark remain.</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="D18" s="114" t="inlineStr">
         <is>
-          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 840/840 with zero required skips/failures/errors.</t>
+          <t>Generated variables separate collected, passed, skipped, failed, and errored statuses; the candidate reports 841/841 with zero required skips/failures/errors.</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="D20" s="114" t="inlineStr">
         <is>
-          <t>Candidate evidence and the clean-clone release package exist with PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
+          <t>Candidate evidence and the clean-clone release package exist with PDF SHA-256 8dc89701bcfb5b4ece4475b4015071470bfc74034f8d85aecd5aa716ea8e4857, JUnit, coverage, variables, figures, expanded manuscript, and a tagged manifest; external release attachment remains open.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="F5" s="114" t="inlineStr">
         <is>
-          <t>Manifest records the v1.4.0-rc19 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records the v1.4.0-rc20 commit/tag, lock/config/source hashes, tools, status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="F6" s="114" t="inlineStr">
         <is>
-          <t>Manifest records tagged v1.4.0-rc19 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
+          <t>Manifest records tagged v1.4.0-rc20 (full revision recorded in the tagged manifest), lock/config/source hashes, tools, clean-clone status, and artifact hashes; shared local unrelated changes remain outside the candidate.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F7" s="114" t="inlineStr">
         <is>
-          <t>Canonical PDF SHA-256 3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d; clean clone at tagged v1.4.0-rc19 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
+          <t>Canonical PDF SHA-256 8dc89701bcfb5b4ece4475b4015071470bfc74034f8d85aecd5aa716ea8e4857; clean clone at tagged v1.4.0-rc20 regenerated the exact PDF, HTML, coverage, JUnit, status, and figure hashes with SOURCE_DATE_EPOCH pinning.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F8" s="114" t="inlineStr">
         <is>
-          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc19; final external publication remains.</t>
+          <t>Candidate source, variables, coverage, JUnit, HTML, PDF, figures, and evidence package were regenerated and verified from tagged v1.4.0-rc20; final external publication remains.</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5228,7 @@
       </c>
       <c r="F16" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected); coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="F17" s="114" t="inlineStr">
         <is>
-          <t>Machine status reports 840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors; pytest collected 841 items and deselected 1; coverage reports exact numerators/denominators.</t>
+          <t>Machine status reports 841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors; pytest collected 841 items and deselected 1; coverage reports exact numerators/denominators.</t>
         </is>
       </c>
     </row>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="F19" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc19 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc20 passed with exact PDF/HTML/evidence/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="F20" s="114" t="inlineStr">
         <is>
-          <t>Clean-clone replay at tagged v1.4.0-rc19 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
+          <t>Clean-clone replay at tagged v1.4.0-rc20 passed with exact PDF/HTML/coverage/JUnit/status/figure hashes; independent reviewer confirmation and external publication remain.</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F24" s="114" t="inlineStr">
         <is>
-          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc19 also passes.</t>
+          <t>Signed strict lifecycle, expiry, tamper, cross-agent, scope, replay, receipt, quarantine, persistence, and concurrency contracts pass; clean-clone replay at v1.4.0-rc20 also passes.</t>
         </is>
       </c>
     </row>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B5" s="117" t="inlineStr">
         <is>
-          <t>v1.4.0-rc19 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
+          <t>v1.4.0-rc20 tagged; clean-clone replay verified; v1.4.0 held pending provider benchmark</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="B7" s="117" t="inlineStr">
         <is>
-          <t>840 JUnit-collected / 840 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected)</t>
+          <t>841 JUnit-collected / 841 passed / 0 skipped / 0 failed / 0 errors (841 pytest items collected; 1 deselected)</t>
         </is>
       </c>
     </row>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="B11" s="117" t="inlineStr">
         <is>
-          <t>3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d</t>
+          <t>8dc89701bcfb5b4ece4475b4015071470bfc74034f8d85aecd5aa716ea8e4857</t>
         </is>
       </c>
     </row>
@@ -5670,7 +5670,7 @@
       </c>
       <c r="B14" s="47" t="inlineStr">
         <is>
-          <t>3e15c79ee15f174bac784a05fa1ebceaed25a8741305f974d51bb3960744503d</t>
+          <t>8dc89701bcfb5b4ece4475b4015071470bfc74034f8d85aecd5aa716ea8e4857</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B15" s="118" t="inlineStr">
         <is>
-          <t>7f42c41a1f42127cf9b06ebc5a53384ecaa5a57fd51a7e2feb84cc0b29999355</t>
+          <t>99846d4132f1a42e59b422f46bc80960cf123ef6f2a527d27a841c7937f55092</t>
         </is>
       </c>
       <c r="C15" s="118" t="n"/>
@@ -5696,7 +5696,7 @@
       </c>
       <c r="B16" s="119" t="inlineStr">
         <is>
-          <t>49ba171b55cd8946d1024dbcbbca12fbe1986e90d3ed152d695c1501f1b44e85</t>
+          <t>b70e43d0785976eeea88c51f2f71a22d13d4e78ac019e19c4c93ce912ba22d63</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="B18" s="119" t="inlineStr">
         <is>
-          <t>cbcfc215fee2cf2200ee0c1ae18e2adf5a2ec9d58c360ef8e691b0b5be963e5eb</t>
+          <t>50f2c14555ec754fdf085fcc7377ad3fa230a8dc93c78ff080b59836801a1d1d</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
       </c>
       <c r="B19" s="119" t="inlineStr">
         <is>
-          <t>fc2f174b03c69d8d3bf038e6e49c11b1c86d39aa74920aa7c226211e6e4a1ecf</t>
+          <t>ce9a8aa6c490a73dc58e53184b6ef19a47cd5be722afc8dd69bd62a5573ed376</t>
         </is>
       </c>
     </row>
@@ -5756,7 +5756,7 @@
       </c>
       <c r="B21" s="119" t="inlineStr">
         <is>
-          <t>fc2f174b03c69d8d3bf038e6e49c11b1c86d39aa74920aa7c226211e6e4a1ecf</t>
+          <t>ce9a8aa6c490a73dc58e53184b6ef19a47cd5be722afc8dd69bd62a5573ed376</t>
         </is>
       </c>
     </row>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="B25" s="119" t="inlineStr">
         <is>
-          <t>Provider-backed run pending; fixture adapter is test-only and cannot produce release evidence</t>
+          <t>Provider-backed run pending; fixture adapter is test-only; independently checked-in executor-key registry is empty awaiting an approved key</t>
         </is>
       </c>
     </row>

</xml_diff>